<commit_message>
update seed data migration with conflict resolution
</commit_message>
<xml_diff>
--- a/src/seed/seed-data/excel/data-seed.xlsx
+++ b/src/seed/seed-data/excel/data-seed.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Robin\Projects\NodeJS\seed-migration-poc\src\seed\seed-data\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{817073E3-0EAB-44BD-96CB-FE269D642140}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD871169-26C2-4248-A81F-954DAAD5F811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{601A8CFE-00A5-4EF9-9576-356BD28C2DB1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{601A8CFE-00A5-4EF9-9576-356BD28C2DB1}"/>
   </bookViews>
   <sheets>
     <sheet name="templates" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="61">
   <si>
     <t>industryId</t>
   </si>
@@ -65,16 +65,10 @@
     <t>approved</t>
   </si>
   <si>
-    <t>Store Audit Template</t>
-  </si>
-  <si>
     <t>published</t>
   </si>
   <si>
     <t>Battery</t>
-  </si>
-  <si>
-    <t>Battery Template</t>
   </si>
   <si>
     <t>Li-ion Battery Template</t>
@@ -155,13 +149,76 @@
   </si>
   <si>
     <t>inputRules</t>
+  </si>
+  <si>
+    <t>Fusing machine</t>
+  </si>
+  <si>
+    <t>Carbon zinc battery Template</t>
+  </si>
+  <si>
+    <t>Gaming Chair</t>
+  </si>
+  <si>
+    <t>temp_uid_1</t>
+  </si>
+  <si>
+    <t>temp_uid_3</t>
+  </si>
+  <si>
+    <t>temp_uid_2</t>
+  </si>
+  <si>
+    <t>temp_uid_4</t>
+  </si>
+  <si>
+    <t>temp_uid_5</t>
+  </si>
+  <si>
+    <t>ind_uid_1</t>
+  </si>
+  <si>
+    <t>ind_uid_2</t>
+  </si>
+  <si>
+    <t>ind_uid_3</t>
+  </si>
+  <si>
+    <t>ind_uid_4</t>
+  </si>
+  <si>
+    <t>ind_uid_5</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>def_Field_uid_1</t>
+  </si>
+  <si>
+    <t>def_Field_uid_2</t>
+  </si>
+  <si>
+    <t>def_Field_uid_3</t>
+  </si>
+  <si>
+    <t>BMW Template</t>
+  </si>
+  <si>
+    <t>Knitting machine</t>
+  </si>
+  <si>
+    <t>def_Field_uid_4</t>
+  </si>
+  <si>
+    <t>Price</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -173,6 +230,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -198,7 +261,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -215,6 +278,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -530,176 +596,263 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FC453D4-8843-4594-B325-C8A1EB3500AF}">
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" customWidth="1"/>
-    <col min="2" max="2" width="13.42578125" customWidth="1"/>
-    <col min="3" max="3" width="28.5703125" customWidth="1"/>
-    <col min="4" max="4" width="14.140625" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" customWidth="1"/>
+    <col min="3" max="3" width="13.42578125" customWidth="1"/>
+    <col min="4" max="4" width="28.5703125" customWidth="1"/>
+    <col min="5" max="5" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
       <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="s">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="2">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2">
+        <v>200</v>
+      </c>
+      <c r="H2" s="2">
+        <v>1</v>
+      </c>
+      <c r="I2" s="2">
+        <v>2</v>
+      </c>
+      <c r="J2" s="2">
+        <v>1</v>
+      </c>
+      <c r="K2" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="E3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" s="2">
+        <v>1</v>
+      </c>
+      <c r="G3" s="2">
+        <v>150</v>
+      </c>
+      <c r="H3" s="2">
+        <v>1</v>
+      </c>
+      <c r="I3" s="2">
+        <v>3</v>
+      </c>
+      <c r="J3" s="2">
+        <v>1</v>
+      </c>
+      <c r="K3" s="2">
         <v>15</v>
       </c>
-      <c r="D2" s="2" t="s">
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="2">
+        <v>1</v>
+      </c>
+      <c r="G4" s="2">
+        <v>300</v>
+      </c>
+      <c r="H4" s="2">
+        <v>1</v>
+      </c>
+      <c r="I4" s="2">
+        <v>4</v>
+      </c>
+      <c r="J4" s="2">
+        <v>1</v>
+      </c>
+      <c r="K4" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="2">
-        <v>1</v>
-      </c>
-      <c r="F2" s="2">
-        <v>200</v>
-      </c>
-      <c r="G2" s="2">
-        <v>1</v>
-      </c>
-      <c r="H2" s="2">
-        <v>2</v>
-      </c>
-      <c r="I2" s="2">
-        <v>1</v>
-      </c>
-      <c r="J2" s="2">
+      <c r="F5" s="2">
+        <v>1</v>
+      </c>
+      <c r="G5" s="2">
+        <v>20</v>
+      </c>
+      <c r="H5" s="2">
+        <v>1</v>
+      </c>
+      <c r="I5" s="2">
+        <v>5</v>
+      </c>
+      <c r="J5" s="2">
+        <v>1</v>
+      </c>
+      <c r="K5" s="2">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="2">
-        <v>1</v>
-      </c>
-      <c r="F3" s="2">
-        <v>150</v>
-      </c>
-      <c r="G3" s="2">
-        <v>1</v>
-      </c>
-      <c r="H3" s="2">
-        <v>3</v>
-      </c>
-      <c r="I3" s="2">
-        <v>1</v>
-      </c>
-      <c r="J3" s="2">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
-        <v>2</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" s="2" t="s">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="2">
+        <v>1</v>
+      </c>
+      <c r="G6" s="2">
+        <v>10</v>
+      </c>
+      <c r="H6" s="2">
+        <v>1</v>
+      </c>
+      <c r="I6" s="2">
+        <v>10</v>
+      </c>
+      <c r="J6" s="2">
+        <v>1</v>
+      </c>
+      <c r="K6" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" s="2">
-        <v>1</v>
-      </c>
-      <c r="F4" s="2">
-        <v>300</v>
-      </c>
-      <c r="G4" s="2">
-        <v>1</v>
-      </c>
-      <c r="H4" s="2">
-        <v>4</v>
-      </c>
-      <c r="I4" s="2">
-        <v>1</v>
-      </c>
-      <c r="J4" s="2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
-        <v>3</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="2" t="s">
+      <c r="F7" s="2">
+        <v>1</v>
+      </c>
+      <c r="G7" s="2">
         <v>10</v>
       </c>
-      <c r="E5" s="2">
-        <v>1</v>
-      </c>
-      <c r="F5" s="2">
-        <v>20</v>
-      </c>
-      <c r="G5" s="2">
-        <v>1</v>
-      </c>
-      <c r="H5" s="2">
-        <v>5</v>
-      </c>
-      <c r="I5" s="2">
-        <v>1</v>
-      </c>
-      <c r="J5" s="2">
+      <c r="H7" s="2">
+        <v>1</v>
+      </c>
+      <c r="I7" s="2">
         <v>10</v>
       </c>
+      <c r="J7" s="2">
+        <v>1</v>
+      </c>
+      <c r="K7" s="2">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="0" r:id="rId1"/>
 </worksheet>
@@ -707,214 +860,297 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19EF8317-8278-4E96-9A13-1F0201354EE4}">
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="26.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>51</v>
+      </c>
+      <c r="B5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B6" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7485ACE2-A2E7-4CDF-BBA7-CA0D03F4EEF8}">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="19.28515625" customWidth="1"/>
-    <col min="3" max="3" width="21" style="4" customWidth="1"/>
-    <col min="4" max="4" width="14.28515625" customWidth="1"/>
-    <col min="5" max="5" width="13.85546875" customWidth="1"/>
-    <col min="6" max="6" width="15.28515625" customWidth="1"/>
-    <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="58.28515625" customWidth="1"/>
-    <col min="9" max="10" width="11.42578125" customWidth="1"/>
-    <col min="11" max="11" width="15.42578125" customWidth="1"/>
-    <col min="12" max="12" width="13.140625" customWidth="1"/>
-    <col min="13" max="13" width="24.85546875" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="21" style="4" customWidth="1"/>
+    <col min="5" max="5" width="14.28515625" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" customWidth="1"/>
+    <col min="7" max="7" width="15.28515625" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1"/>
+    <col min="9" max="9" width="58.28515625" customWidth="1"/>
+    <col min="10" max="11" width="11.42578125" customWidth="1"/>
+    <col min="12" max="12" width="15.42578125" customWidth="1"/>
+    <col min="13" max="13" width="13.140625" customWidth="1"/>
+    <col min="14" max="14" width="24.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="G1" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="N1" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="90" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="K1" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1" s="5" t="s">
+      <c r="D2" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" ht="90" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
+      <c r="G2" t="s">
+        <v>30</v>
+      </c>
+      <c r="I2" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="J2" t="s">
+        <v>38</v>
+      </c>
+      <c r="K2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M2" t="b">
+        <v>1</v>
+      </c>
+      <c r="N2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="105" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C3">
+        <v>3</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3">
         <v>2</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="F3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" t="s">
         <v>30</v>
       </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F2" t="s">
-        <v>32</v>
-      </c>
-      <c r="H2" s="4" t="s">
+      <c r="I3" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="I2" t="s">
-        <v>40</v>
-      </c>
-      <c r="J2" t="s">
-        <v>40</v>
-      </c>
-      <c r="K2" t="b">
-        <v>1</v>
-      </c>
-      <c r="L2" t="b">
-        <v>1</v>
-      </c>
-      <c r="M2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" ht="105" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>1</v>
-      </c>
-      <c r="B3">
+      <c r="J3" t="s">
+        <v>38</v>
+      </c>
+      <c r="K3" t="s">
+        <v>38</v>
+      </c>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
+      <c r="M3" t="b">
+        <v>0</v>
+      </c>
+      <c r="N3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4">
+        <v>4</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4">
         <v>3</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="D3">
-        <v>2</v>
-      </c>
-      <c r="E3" t="s">
-        <v>31</v>
-      </c>
-      <c r="F3" t="s">
-        <v>32</v>
-      </c>
-      <c r="H3" s="4" t="s">
+      <c r="F4" t="s">
         <v>35</v>
       </c>
-      <c r="I3" t="s">
-        <v>40</v>
-      </c>
-      <c r="J3" t="s">
-        <v>40</v>
-      </c>
-      <c r="K3" t="b">
-        <v>1</v>
-      </c>
-      <c r="L3" t="b">
+      <c r="G4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="J4" t="s">
+        <v>38</v>
+      </c>
+      <c r="K4" t="s">
+        <v>38</v>
+      </c>
+      <c r="L4" t="b">
         <v>0</v>
       </c>
-      <c r="M3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" ht="60" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>2</v>
-      </c>
-      <c r="B4">
+      <c r="M4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5">
+        <v>5</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="E5">
         <v>4</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="F5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4" t="s">
-        <v>37</v>
-      </c>
-      <c r="F4" t="s">
-        <v>32</v>
-      </c>
-      <c r="H4" s="4" t="s">
+      <c r="J5" t="s">
         <v>38</v>
       </c>
-      <c r="I4" t="s">
-        <v>40</v>
-      </c>
-      <c r="J4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K4" t="b">
-        <v>0</v>
-      </c>
-      <c r="L4" t="b">
-        <v>1</v>
-      </c>
-      <c r="M4" t="b">
-        <v>0</v>
+      <c r="K5" t="s">
+        <v>38</v>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M5" t="b">
+        <v>1</v>
+      </c>
+      <c r="N5" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
prepare seed version and checksum compare
</commit_message>
<xml_diff>
--- a/src/seed/seed-data/excel/data-seed.xlsx
+++ b/src/seed/seed-data/excel/data-seed.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Robin\Projects\NodeJS\seed-migration-poc\src\seed\seed-data\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD871169-26C2-4248-A81F-954DAAD5F811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B983D4B7-C188-431D-B268-4F1DD71A0863}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{601A8CFE-00A5-4EF9-9576-356BD28C2DB1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{601A8CFE-00A5-4EF9-9576-356BD28C2DB1}"/>
   </bookViews>
   <sheets>
     <sheet name="templates" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="62">
   <si>
     <t>industryId</t>
   </si>
@@ -211,7 +211,10 @@
     <t>def_Field_uid_4</t>
   </si>
   <si>
-    <t>Price</t>
+    <t>temp_uid_6</t>
+  </si>
+  <si>
+    <t>Product Price</t>
   </si>
 </sst>
 </file>
@@ -818,7 +821,7 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="B7" t="s">
         <v>51</v>
@@ -1119,7 +1122,7 @@
         <v>5</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E5">
         <v>4</v>

</xml_diff>

<commit_message>
file hash check before db operation
</commit_message>
<xml_diff>
--- a/src/seed/seed-data/excel/data-seed.xlsx
+++ b/src/seed/seed-data/excel/data-seed.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Robin\Projects\NodeJS\seed-migration-poc\src\seed\seed-data\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B983D4B7-C188-431D-B268-4F1DD71A0863}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B04B89BE-3123-40BE-81EC-58BB4624D9EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{601A8CFE-00A5-4EF9-9576-356BD28C2DB1}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="67">
   <si>
     <t>industryId</t>
   </si>
@@ -157,9 +157,6 @@
     <t>Carbon zinc battery Template</t>
   </si>
   <si>
-    <t>Gaming Chair</t>
-  </si>
-  <si>
     <t>temp_uid_1</t>
   </si>
   <si>
@@ -215,6 +212,24 @@
   </si>
   <si>
     <t>Product Price</t>
+  </si>
+  <si>
+    <t>Wind Turbine</t>
+  </si>
+  <si>
+    <t>temp_uid_7</t>
+  </si>
+  <si>
+    <t>Audi Template</t>
+  </si>
+  <si>
+    <t>def_Field_uid_5</t>
+  </si>
+  <si>
+    <t>decimal</t>
+  </si>
+  <si>
+    <t>Product Base Price</t>
   </si>
 </sst>
 </file>
@@ -599,7 +614,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FC453D4-8843-4594-B325-C8A1EB3500AF}">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
@@ -611,7 +626,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -646,10 +661,10 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>13</v>
@@ -681,10 +696,10 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>13</v>
@@ -716,16 +731,16 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>12</v>
@@ -751,10 +766,10 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>15</v>
@@ -786,10 +801,10 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>18</v>
@@ -821,16 +836,16 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>18</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>12</v>
@@ -851,6 +866,41 @@
         <v>1</v>
       </c>
       <c r="K7" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>62</v>
+      </c>
+      <c r="B8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="2">
+        <v>1</v>
+      </c>
+      <c r="G8" s="2">
+        <v>25</v>
+      </c>
+      <c r="H8" s="2">
+        <v>1</v>
+      </c>
+      <c r="I8" s="2">
+        <v>5</v>
+      </c>
+      <c r="J8" s="2">
+        <v>1</v>
+      </c>
+      <c r="K8" s="2">
         <v>10</v>
       </c>
     </row>
@@ -872,7 +922,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>2</v>
@@ -880,7 +930,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
         <v>13</v>
@@ -888,7 +938,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
         <v>17</v>
@@ -896,7 +946,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
         <v>15</v>
@@ -904,7 +954,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
         <v>18</v>
@@ -912,10 +962,10 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -926,7 +976,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7485ACE2-A2E7-4CDF-BBA7-CA0D03F4EEF8}">
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
@@ -946,7 +996,7 @@
   <sheetData>
     <row r="1" spans="1:14" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>0</v>
@@ -990,10 +1040,10 @@
     </row>
     <row r="2" spans="1:14" ht="90" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C2">
         <v>2</v>
@@ -1031,10 +1081,10 @@
     </row>
     <row r="3" spans="1:14" ht="105" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C3">
         <v>3</v>
@@ -1072,10 +1122,10 @@
     </row>
     <row r="4" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C4">
         <v>4</v>
@@ -1113,16 +1163,16 @@
     </row>
     <row r="5" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C5">
         <v>5</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -1149,6 +1199,47 @@
         <v>1</v>
       </c>
       <c r="N5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" ht="105" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6" t="s">
+        <v>65</v>
+      </c>
+      <c r="G6" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" t="s">
+        <v>38</v>
+      </c>
+      <c r="K6" t="s">
+        <v>38</v>
+      </c>
+      <c r="L6" t="b">
+        <v>1</v>
+      </c>
+      <c r="M6" t="b">
+        <v>1</v>
+      </c>
+      <c r="N6" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
detect excel data change before converting to json
</commit_message>
<xml_diff>
--- a/src/seed/seed-data/excel/data-seed.xlsx
+++ b/src/seed/seed-data/excel/data-seed.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Robin\Projects\NodeJS\seed-migration-poc\src\seed\seed-data\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B04B89BE-3123-40BE-81EC-58BB4624D9EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63F01E6F-58D8-499F-BFBA-40F7AE5130AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{601A8CFE-00A5-4EF9-9576-356BD28C2DB1}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="72">
   <si>
     <t>industryId</t>
   </si>
@@ -220,16 +220,31 @@
     <t>temp_uid_7</t>
   </si>
   <si>
-    <t>Audi Template</t>
-  </si>
-  <si>
     <t>def_Field_uid_5</t>
   </si>
   <si>
-    <t>decimal</t>
-  </si>
-  <si>
     <t>Product Base Price</t>
+  </si>
+  <si>
+    <t>environment</t>
+  </si>
+  <si>
+    <t>dev</t>
+  </si>
+  <si>
+    <t>staging</t>
+  </si>
+  <si>
+    <t>{}</t>
+  </si>
+  <si>
+    <t>Base Car template</t>
+  </si>
+  <si>
+    <t>def_Field_uid_6</t>
+  </si>
+  <si>
+    <t>Model</t>
   </si>
 </sst>
 </file>
@@ -614,7 +629,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FC453D4-8843-4594-B325-C8A1EB3500AF}">
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" bestFit="1" customWidth="1"/>
@@ -622,9 +637,10 @@
     <col min="3" max="3" width="13.42578125" customWidth="1"/>
     <col min="4" max="4" width="28.5703125" customWidth="1"/>
     <col min="5" max="5" width="14.140625" customWidth="1"/>
+    <col min="12" max="12" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>52</v>
       </c>
@@ -658,8 +674,11 @@
       <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L1" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>42</v>
       </c>
@@ -693,8 +712,11 @@
       <c r="K2" s="2">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>44</v>
       </c>
@@ -729,7 +751,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>43</v>
       </c>
@@ -763,8 +785,11 @@
       <c r="K4" s="2">
         <v>20</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>45</v>
       </c>
@@ -799,7 +824,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>46</v>
       </c>
@@ -834,7 +859,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>59</v>
       </c>
@@ -869,7 +894,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>62</v>
       </c>
@@ -880,7 +905,7 @@
         <v>17</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>10</v>
@@ -895,13 +920,13 @@
         <v>1</v>
       </c>
       <c r="I8" s="2">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="J8" s="2">
         <v>1</v>
       </c>
       <c r="K8" s="2">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -976,7 +1001,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7485ACE2-A2E7-4CDF-BBA7-CA0D03F4EEF8}">
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
@@ -1060,6 +1085,9 @@
       <c r="G2" t="s">
         <v>30</v>
       </c>
+      <c r="H2" t="s">
+        <v>68</v>
+      </c>
       <c r="I2" s="4" t="s">
         <v>31</v>
       </c>
@@ -1101,6 +1129,9 @@
       <c r="G3" t="s">
         <v>30</v>
       </c>
+      <c r="H3" t="s">
+        <v>68</v>
+      </c>
       <c r="I3" s="4" t="s">
         <v>33</v>
       </c>
@@ -1142,6 +1173,9 @@
       <c r="G4" t="s">
         <v>30</v>
       </c>
+      <c r="H4" t="s">
+        <v>68</v>
+      </c>
       <c r="I4" s="4" t="s">
         <v>36</v>
       </c>
@@ -1183,6 +1217,9 @@
       <c r="G5" t="s">
         <v>30</v>
       </c>
+      <c r="H5" t="s">
+        <v>68</v>
+      </c>
       <c r="I5" s="4" t="s">
         <v>36</v>
       </c>
@@ -1204,7 +1241,7 @@
     </row>
     <row r="6" spans="1:14" ht="105" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B6" t="s">
         <v>48</v>
@@ -1213,17 +1250,17 @@
         <v>5</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E6">
         <v>5</v>
       </c>
-      <c r="F6" t="s">
-        <v>65</v>
-      </c>
       <c r="G6" t="s">
         <v>30</v>
       </c>
+      <c r="H6" t="s">
+        <v>68</v>
+      </c>
       <c r="I6" s="4" t="s">
         <v>33</v>
       </c>
@@ -1240,6 +1277,44 @@
         <v>1</v>
       </c>
       <c r="N6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" ht="105" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7">
+        <v>5</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="E7">
+        <v>6</v>
+      </c>
+      <c r="F7" t="s">
+        <v>29</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="J7" t="s">
+        <v>38</v>
+      </c>
+      <c r="K7" t="s">
+        <v>38</v>
+      </c>
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
+      <c r="M7" t="b">
+        <v>1</v>
+      </c>
+      <c r="N7" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
load seed data json with env overrides
</commit_message>
<xml_diff>
--- a/src/seed/seed-data/excel/data-seed.xlsx
+++ b/src/seed/seed-data/excel/data-seed.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="80">
   <si>
     <t>id</t>
   </si>
@@ -141,16 +141,25 @@
     <t>Base Car template</t>
   </si>
   <si>
+    <t>temp_uid_8</t>
+  </si>
+  <si>
+    <t>ind_uid_6</t>
+  </si>
+  <si>
+    <t>Footware</t>
+  </si>
+  <si>
+    <t>Base Footware Template</t>
+  </si>
+  <si>
+    <t>Staging</t>
+  </si>
+  <si>
     <t>ind_uid_5</t>
   </si>
   <si>
     <t>Wind Turbine</t>
-  </si>
-  <si>
-    <t>ind_uid_6</t>
-  </si>
-  <si>
-    <t>Footware</t>
   </si>
   <si>
     <t>defaultSectionId</t>
@@ -346,6 +355,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -357,9 +369,6 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
@@ -1746,19 +1755,45 @@
       </c>
     </row>
     <row r="9" ht="13.55" customHeight="1">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
-      <c r="J9" s="7"/>
-      <c r="K9" s="7"/>
-      <c r="L9" s="7"/>
-      <c r="M9" s="7"/>
+      <c r="A9" t="s" s="4">
+        <v>42</v>
+      </c>
+      <c r="B9" t="s" s="4">
+        <v>43</v>
+      </c>
+      <c r="C9" t="s" s="4">
+        <v>44</v>
+      </c>
+      <c r="D9" t="s" s="4">
+        <v>45</v>
+      </c>
+      <c r="E9" t="s" s="4">
+        <v>22</v>
+      </c>
+      <c r="F9" s="8">
+        <v>1</v>
+      </c>
+      <c r="G9" s="8">
+        <v>15</v>
+      </c>
+      <c r="H9" s="8">
+        <v>1</v>
+      </c>
+      <c r="I9" s="8">
+        <v>10</v>
+      </c>
+      <c r="J9" s="8">
+        <v>1</v>
+      </c>
+      <c r="K9" s="8">
+        <v>20</v>
+      </c>
+      <c r="L9" t="s" s="4">
+        <v>28</v>
+      </c>
+      <c r="M9" t="s" s="4">
+        <v>19</v>
+      </c>
     </row>
     <row r="10" ht="13.55" customHeight="1">
       <c r="A10" s="7"/>
@@ -1786,126 +1821,136 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E10"/>
+  <dimension ref="B2:F11"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="15" style="8" customWidth="1"/>
-    <col min="2" max="2" width="26.6719" style="8" customWidth="1"/>
-    <col min="3" max="5" width="8.85156" style="8" customWidth="1"/>
-    <col min="6" max="16384" width="8.85156" style="8" customWidth="1"/>
+    <col min="1" max="1" width="11.0703" style="9" customWidth="1"/>
+    <col min="2" max="2" width="15" style="9" customWidth="1"/>
+    <col min="3" max="3" width="26.6719" style="9" customWidth="1"/>
+    <col min="4" max="4" width="8.85156" style="9" customWidth="1"/>
+    <col min="5" max="5" width="12.6797" style="9" customWidth="1"/>
+    <col min="6" max="6" width="8.85156" style="9" customWidth="1"/>
+    <col min="7" max="16384" width="8.85156" style="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13.55" customHeight="1">
-      <c r="A1" t="s" s="9">
+    <row r="1" ht="45.6" customHeight="1"/>
+    <row r="2" ht="13.55" customHeight="1">
+      <c r="B2" t="s" s="10">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="9">
+      <c r="C2" t="s" s="10">
         <v>3</v>
       </c>
-      <c r="C1" t="s" s="4">
+      <c r="D2" t="s" s="10">
         <v>12</v>
       </c>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-    </row>
-    <row r="2" ht="13.55" customHeight="1">
-      <c r="A2" t="s" s="4">
+      <c r="E2" t="s" s="10">
+        <v>11</v>
+      </c>
+      <c r="F2" s="7"/>
+    </row>
+    <row r="3" ht="13.55" customHeight="1">
+      <c r="B3" t="s" s="4">
         <v>14</v>
       </c>
-      <c r="B2" t="s" s="4">
+      <c r="C3" t="s" s="4">
         <v>15</v>
       </c>
-      <c r="C2" t="s" s="4">
+      <c r="D3" t="s" s="4">
+        <v>19</v>
+      </c>
+      <c r="E3" t="s" s="4">
+        <v>28</v>
+      </c>
+      <c r="F3" s="7"/>
+    </row>
+    <row r="4" ht="13.55" customHeight="1">
+      <c r="B4" t="s" s="4">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s" s="4">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s" s="4">
         <v>29</v>
       </c>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-    </row>
-    <row r="3" ht="13.55" customHeight="1">
-      <c r="A3" t="s" s="4">
-        <v>24</v>
-      </c>
-      <c r="B3" t="s" s="4">
-        <v>25</v>
-      </c>
-      <c r="C3" t="s" s="4">
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+    </row>
+    <row r="5" ht="13.55" customHeight="1">
+      <c r="B5" t="s" s="4">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s" s="4">
+        <v>32</v>
+      </c>
+      <c r="D5" t="s" s="4">
+        <v>19</v>
+      </c>
+      <c r="E5" t="s" s="4">
+        <v>46</v>
+      </c>
+      <c r="F5" s="7"/>
+    </row>
+    <row r="6" ht="13.55" customHeight="1">
+      <c r="B6" t="s" s="4">
+        <v>35</v>
+      </c>
+      <c r="C6" t="s" s="4">
+        <v>36</v>
+      </c>
+      <c r="D6" t="s" s="4">
         <v>29</v>
       </c>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-    </row>
-    <row r="4" ht="13.55" customHeight="1">
-      <c r="A4" t="s" s="4">
-        <v>31</v>
-      </c>
-      <c r="B4" t="s" s="4">
-        <v>32</v>
-      </c>
-      <c r="C4" t="s" s="4">
-        <v>19</v>
-      </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-    </row>
-    <row r="5" ht="13.55" customHeight="1">
-      <c r="A5" t="s" s="4">
-        <v>35</v>
-      </c>
-      <c r="B5" t="s" s="4">
-        <v>36</v>
-      </c>
-      <c r="C5" t="s" s="4">
+      <c r="E6" s="7"/>
+      <c r="F6" s="7"/>
+    </row>
+    <row r="7" ht="13.55" customHeight="1">
+      <c r="B7" t="s" s="4">
+        <v>47</v>
+      </c>
+      <c r="C7" t="s" s="4">
+        <v>48</v>
+      </c>
+      <c r="D7" t="s" s="4">
         <v>29</v>
       </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-    </row>
-    <row r="6" ht="13.55" customHeight="1">
-      <c r="A6" t="s" s="4">
-        <v>42</v>
-      </c>
-      <c r="B6" t="s" s="4">
+      <c r="E7" s="7"/>
+      <c r="F7" s="7"/>
+    </row>
+    <row r="8" ht="13.55" customHeight="1">
+      <c r="B8" t="s" s="4">
         <v>43</v>
       </c>
-      <c r="C6" t="s" s="4">
+      <c r="C8" t="s" s="4">
+        <v>44</v>
+      </c>
+      <c r="D8" t="s" s="4">
         <v>29</v>
       </c>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-    </row>
-    <row r="7" ht="13.55" customHeight="1">
-      <c r="A7" t="s" s="4">
-        <v>44</v>
-      </c>
-      <c r="B7" t="s" s="4">
-        <v>45</v>
-      </c>
-      <c r="C7" t="s" s="4">
-        <v>19</v>
-      </c>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-    </row>
-    <row r="8" ht="13.55" customHeight="1">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
       <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
     </row>
     <row r="9" ht="13.55" customHeight="1">
-      <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
     </row>
     <row r="10" ht="13.55" customHeight="1">
-      <c r="A10" s="7"/>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
       <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+    </row>
+    <row r="11" ht="13.55" customHeight="1">
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1921,20 +1966,20 @@
   <dimension ref="A1:O10"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="15.5" style="10" customWidth="1"/>
-    <col min="2" max="2" width="14" style="10" customWidth="1"/>
-    <col min="3" max="3" width="19.3516" style="10" customWidth="1"/>
-    <col min="4" max="4" width="21" style="10" customWidth="1"/>
-    <col min="5" max="5" width="14.3516" style="10" customWidth="1"/>
-    <col min="6" max="6" width="13.8516" style="10" customWidth="1"/>
-    <col min="7" max="7" width="15.3516" style="10" customWidth="1"/>
-    <col min="8" max="8" width="15" style="10" customWidth="1"/>
-    <col min="9" max="9" width="58.3516" style="10" customWidth="1"/>
-    <col min="10" max="11" width="11.5" style="10" customWidth="1"/>
-    <col min="12" max="12" width="15.5" style="10" customWidth="1"/>
-    <col min="13" max="13" width="13.1719" style="10" customWidth="1"/>
-    <col min="14" max="15" width="24.8516" style="10" customWidth="1"/>
-    <col min="16" max="16384" width="8.85156" style="10" customWidth="1"/>
+    <col min="1" max="1" width="15.5" style="11" customWidth="1"/>
+    <col min="2" max="2" width="14" style="11" customWidth="1"/>
+    <col min="3" max="3" width="19.3516" style="11" customWidth="1"/>
+    <col min="4" max="4" width="21" style="11" customWidth="1"/>
+    <col min="5" max="5" width="14.3516" style="11" customWidth="1"/>
+    <col min="6" max="6" width="13.8516" style="11" customWidth="1"/>
+    <col min="7" max="7" width="15.3516" style="11" customWidth="1"/>
+    <col min="8" max="8" width="15" style="11" customWidth="1"/>
+    <col min="9" max="9" width="58.3516" style="11" customWidth="1"/>
+    <col min="10" max="11" width="11.5" style="11" customWidth="1"/>
+    <col min="12" max="12" width="15.5" style="11" customWidth="1"/>
+    <col min="13" max="13" width="13.1719" style="11" customWidth="1"/>
+    <col min="14" max="15" width="24.8516" style="11" customWidth="1"/>
+    <col min="16" max="16384" width="8.85156" style="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="13.55" customHeight="1">
@@ -1945,40 +1990,40 @@
         <v>1</v>
       </c>
       <c r="C1" t="s" s="4">
-        <v>46</v>
-      </c>
-      <c r="D1" t="s" s="11">
+        <v>49</v>
+      </c>
+      <c r="D1" t="s" s="12">
         <v>3</v>
       </c>
       <c r="E1" t="s" s="4">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="F1" t="s" s="4">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="G1" t="s" s="4">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="H1" t="s" s="4">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="I1" t="s" s="4">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="J1" t="s" s="4">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="K1" t="s" s="4">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="L1" t="s" s="4">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="M1" t="s" s="4">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="N1" t="s" s="4">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="O1" t="s" s="4">
         <v>12</v>
@@ -1986,45 +2031,45 @@
     </row>
     <row r="2" ht="90" customHeight="1">
       <c r="A2" t="s" s="4">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B2" t="s" s="4">
         <v>14</v>
       </c>
-      <c r="C2" s="12">
+      <c r="C2" s="8">
         <v>2</v>
       </c>
-      <c r="D2" t="s" s="11">
-        <v>58</v>
-      </c>
-      <c r="E2" s="12">
+      <c r="D2" t="s" s="12">
+        <v>61</v>
+      </c>
+      <c r="E2" s="8">
         <v>1</v>
       </c>
       <c r="F2" t="s" s="4">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G2" t="s" s="4">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="H2" t="s" s="4">
-        <v>61</v>
-      </c>
-      <c r="I2" t="s" s="11">
-        <v>62</v>
+        <v>64</v>
+      </c>
+      <c r="I2" t="s" s="12">
+        <v>65</v>
       </c>
       <c r="J2" t="s" s="4">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K2" t="s" s="4">
-        <v>63</v>
-      </c>
-      <c r="L2" t="b" s="12">
-        <v>1</v>
-      </c>
-      <c r="M2" t="b" s="12">
-        <v>1</v>
-      </c>
-      <c r="N2" t="b" s="12">
+        <v>66</v>
+      </c>
+      <c r="L2" t="b" s="8">
+        <v>1</v>
+      </c>
+      <c r="M2" t="b" s="8">
+        <v>1</v>
+      </c>
+      <c r="N2" t="b" s="8">
         <v>1</v>
       </c>
       <c r="O2" t="s" s="4">
@@ -2033,45 +2078,45 @@
     </row>
     <row r="3" ht="105" customHeight="1">
       <c r="A3" t="s" s="4">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B3" t="s" s="4">
         <v>14</v>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="8">
         <v>3</v>
       </c>
-      <c r="D3" t="s" s="11">
-        <v>65</v>
-      </c>
-      <c r="E3" s="12">
+      <c r="D3" t="s" s="12">
+        <v>68</v>
+      </c>
+      <c r="E3" s="8">
         <v>2</v>
       </c>
       <c r="F3" t="s" s="4">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G3" t="s" s="4">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="H3" t="s" s="4">
-        <v>61</v>
-      </c>
-      <c r="I3" t="s" s="11">
+        <v>64</v>
+      </c>
+      <c r="I3" t="s" s="12">
+        <v>69</v>
+      </c>
+      <c r="J3" t="s" s="4">
         <v>66</v>
       </c>
-      <c r="J3" t="s" s="4">
-        <v>63</v>
-      </c>
       <c r="K3" t="s" s="4">
-        <v>63</v>
-      </c>
-      <c r="L3" t="b" s="12">
-        <v>1</v>
-      </c>
-      <c r="M3" t="b" s="12">
+        <v>66</v>
+      </c>
+      <c r="L3" t="b" s="8">
+        <v>1</v>
+      </c>
+      <c r="M3" t="b" s="8">
         <v>0</v>
       </c>
-      <c r="N3" t="b" s="12">
+      <c r="N3" t="b" s="8">
         <v>1</v>
       </c>
       <c r="O3" t="s" s="4">
@@ -2080,45 +2125,45 @@
     </row>
     <row r="4" ht="60" customHeight="1">
       <c r="A4" t="s" s="4">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B4" t="s" s="4">
         <v>24</v>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="8">
         <v>4</v>
       </c>
-      <c r="D4" t="s" s="11">
-        <v>68</v>
-      </c>
-      <c r="E4" s="12">
+      <c r="D4" t="s" s="12">
+        <v>71</v>
+      </c>
+      <c r="E4" s="8">
         <v>3</v>
       </c>
       <c r="F4" t="s" s="4">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G4" t="s" s="4">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="H4" t="s" s="4">
-        <v>61</v>
-      </c>
-      <c r="I4" t="s" s="11">
-        <v>70</v>
+        <v>64</v>
+      </c>
+      <c r="I4" t="s" s="12">
+        <v>73</v>
       </c>
       <c r="J4" t="s" s="4">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K4" t="s" s="4">
-        <v>63</v>
-      </c>
-      <c r="L4" t="b" s="12">
+        <v>66</v>
+      </c>
+      <c r="L4" t="b" s="8">
         <v>0</v>
       </c>
-      <c r="M4" t="b" s="12">
-        <v>1</v>
-      </c>
-      <c r="N4" t="b" s="12">
+      <c r="M4" t="b" s="8">
+        <v>1</v>
+      </c>
+      <c r="N4" t="b" s="8">
         <v>0</v>
       </c>
       <c r="O4" t="s" s="4">
@@ -2127,45 +2172,45 @@
     </row>
     <row r="5" ht="60" customHeight="1">
       <c r="A5" t="s" s="4">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B5" t="s" s="4">
         <v>24</v>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="8">
         <v>5</v>
       </c>
-      <c r="D5" t="s" s="11">
-        <v>72</v>
-      </c>
-      <c r="E5" s="12">
+      <c r="D5" t="s" s="12">
+        <v>75</v>
+      </c>
+      <c r="E5" s="8">
         <v>4</v>
       </c>
       <c r="F5" t="s" s="4">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G5" t="s" s="4">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="H5" t="s" s="4">
-        <v>61</v>
-      </c>
-      <c r="I5" t="s" s="11">
-        <v>70</v>
+        <v>64</v>
+      </c>
+      <c r="I5" t="s" s="12">
+        <v>73</v>
       </c>
       <c r="J5" t="s" s="4">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="K5" t="s" s="4">
-        <v>63</v>
-      </c>
-      <c r="L5" t="b" s="12">
-        <v>1</v>
-      </c>
-      <c r="M5" t="b" s="12">
-        <v>1</v>
-      </c>
-      <c r="N5" t="b" s="12">
+        <v>66</v>
+      </c>
+      <c r="L5" t="b" s="8">
+        <v>1</v>
+      </c>
+      <c r="M5" t="b" s="8">
+        <v>1</v>
+      </c>
+      <c r="N5" t="b" s="8">
         <v>1</v>
       </c>
       <c r="O5" t="s" s="4">
@@ -2174,43 +2219,43 @@
     </row>
     <row r="6" ht="105" customHeight="1">
       <c r="A6" t="s" s="4">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B6" t="s" s="4">
         <v>24</v>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="8">
         <v>5</v>
       </c>
-      <c r="D6" t="s" s="11">
-        <v>74</v>
-      </c>
-      <c r="E6" s="12">
+      <c r="D6" t="s" s="12">
+        <v>77</v>
+      </c>
+      <c r="E6" s="8">
         <v>5</v>
       </c>
       <c r="F6" s="7"/>
       <c r="G6" t="s" s="4">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="H6" t="s" s="4">
-        <v>61</v>
-      </c>
-      <c r="I6" t="s" s="11">
+        <v>64</v>
+      </c>
+      <c r="I6" t="s" s="12">
+        <v>69</v>
+      </c>
+      <c r="J6" t="s" s="4">
         <v>66</v>
       </c>
-      <c r="J6" t="s" s="4">
-        <v>63</v>
-      </c>
       <c r="K6" t="s" s="4">
-        <v>63</v>
-      </c>
-      <c r="L6" t="b" s="12">
-        <v>1</v>
-      </c>
-      <c r="M6" t="b" s="12">
-        <v>1</v>
-      </c>
-      <c r="N6" t="b" s="12">
+        <v>66</v>
+      </c>
+      <c r="L6" t="b" s="8">
+        <v>1</v>
+      </c>
+      <c r="M6" t="b" s="8">
+        <v>1</v>
+      </c>
+      <c r="N6" t="b" s="8">
         <v>1</v>
       </c>
       <c r="O6" t="s" s="4">
@@ -2219,41 +2264,41 @@
     </row>
     <row r="7" ht="105" customHeight="1">
       <c r="A7" t="s" s="4">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B7" t="s" s="4">
         <v>24</v>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="8">
         <v>5</v>
       </c>
-      <c r="D7" t="s" s="11">
-        <v>76</v>
-      </c>
-      <c r="E7" s="12">
+      <c r="D7" t="s" s="12">
+        <v>79</v>
+      </c>
+      <c r="E7" s="8">
         <v>6</v>
       </c>
       <c r="F7" t="s" s="4">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G7" s="7"/>
       <c r="H7" s="7"/>
-      <c r="I7" t="s" s="11">
+      <c r="I7" t="s" s="12">
+        <v>69</v>
+      </c>
+      <c r="J7" t="s" s="4">
         <v>66</v>
       </c>
-      <c r="J7" t="s" s="4">
-        <v>63</v>
-      </c>
       <c r="K7" t="s" s="4">
-        <v>63</v>
-      </c>
-      <c r="L7" t="b" s="12">
-        <v>1</v>
-      </c>
-      <c r="M7" t="b" s="12">
-        <v>1</v>
-      </c>
-      <c r="N7" t="b" s="12">
+        <v>66</v>
+      </c>
+      <c r="L7" t="b" s="8">
+        <v>1</v>
+      </c>
+      <c r="M7" t="b" s="8">
+        <v>1</v>
+      </c>
+      <c r="N7" t="b" s="8">
         <v>1</v>
       </c>
       <c r="O7" t="s" s="4">

</xml_diff>

<commit_message>
remove base json and generated env specific json only
</commit_message>
<xml_diff>
--- a/src/seed/seed-data/excel/data-seed.xlsx
+++ b/src/seed/seed-data/excel/data-seed.xlsx
@@ -5,9 +5,9 @@
     <workbookView xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080"/>
   </bookViews>
   <sheets>
-    <sheet name="templates" sheetId="1" r:id="rId4"/>
-    <sheet name="industries" sheetId="2" r:id="rId5"/>
-    <sheet name="default_fields" sheetId="3" r:id="rId6"/>
+    <sheet name="industries" sheetId="1" r:id="rId4"/>
+    <sheet name="templates" sheetId="2" r:id="rId5"/>
+    <sheet name="defaultFields" sheetId="3" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -18,15 +18,72 @@
     <t>id</t>
   </si>
   <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>priority</t>
+  </si>
+  <si>
+    <t>environment</t>
+  </si>
+  <si>
+    <t>ind_uid_1</t>
+  </si>
+  <si>
+    <t>Battery</t>
+  </si>
+  <si>
+    <t>DB</t>
+  </si>
+  <si>
+    <t>local,dev,staging</t>
+  </si>
+  <si>
+    <t>ind_uid_2</t>
+  </si>
+  <si>
+    <t>Automotive</t>
+  </si>
+  <si>
+    <t>SEED</t>
+  </si>
+  <si>
+    <t>local,dev</t>
+  </si>
+  <si>
+    <t>ind_uid_3</t>
+  </si>
+  <si>
+    <t>Furniture</t>
+  </si>
+  <si>
+    <t>local,staging</t>
+  </si>
+  <si>
+    <t>ind_uid_4</t>
+  </si>
+  <si>
+    <t>Textile</t>
+  </si>
+  <si>
+    <t>ind_uid_5</t>
+  </si>
+  <si>
+    <t>Wind Turbine Tech</t>
+  </si>
+  <si>
+    <t>ind_uid_6</t>
+  </si>
+  <si>
+    <t>Footwear</t>
+  </si>
+  <si>
     <t>industryId</t>
   </si>
   <si>
     <t>industryName</t>
   </si>
   <si>
-    <t>name</t>
-  </si>
-  <si>
     <t>status</t>
   </si>
   <si>
@@ -48,33 +105,15 @@
     <t>maxSections</t>
   </si>
   <si>
-    <t>environment</t>
-  </si>
-  <si>
-    <t>priority</t>
-  </si>
-  <si>
     <t>temp_uid_1</t>
   </si>
   <si>
-    <t>ind_uid_1</t>
-  </si>
-  <si>
-    <t>Battery</t>
-  </si>
-  <si>
     <t>Carbon zinc battery Template</t>
   </si>
   <si>
     <t>draft</t>
   </si>
   <si>
-    <t>dev</t>
-  </si>
-  <si>
-    <t>DB</t>
-  </si>
-  <si>
     <t>temp_uid_2</t>
   </si>
   <si>
@@ -87,45 +126,21 @@
     <t>temp_uid_3</t>
   </si>
   <si>
-    <t>ind_uid_2</t>
-  </si>
-  <si>
-    <t>Automotive</t>
-  </si>
-  <si>
     <t>BMW Template</t>
   </si>
   <si>
     <t>published</t>
   </si>
   <si>
-    <t>staging</t>
-  </si>
-  <si>
-    <t>SEED</t>
-  </si>
-  <si>
     <t>temp_uid_4</t>
   </si>
   <si>
-    <t>ind_uid_3</t>
-  </si>
-  <si>
-    <t>Furniture</t>
-  </si>
-  <si>
     <t>Furniture Tech Template</t>
   </si>
   <si>
     <t>temp_uid_5</t>
   </si>
   <si>
-    <t>ind_uid_4</t>
-  </si>
-  <si>
-    <t>Textile</t>
-  </si>
-  <si>
     <t>Fusing machine</t>
   </si>
   <si>
@@ -144,25 +159,10 @@
     <t>temp_uid_8</t>
   </si>
   <si>
-    <t>ind_uid_6</t>
-  </si>
-  <si>
     <t>Footware</t>
   </si>
   <si>
     <t>Base Footware Template</t>
-  </si>
-  <si>
-    <t>Staging</t>
-  </si>
-  <si>
-    <t>ind_uid_5</t>
-  </si>
-  <si>
-    <t>Wind Turbine Tech</t>
-  </si>
-  <si>
-    <t>Footwear</t>
   </si>
   <si>
     <t>defaultSectionId</t>
@@ -333,8 +333,20 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
@@ -347,16 +359,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
@@ -364,14 +370,11 @@
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
@@ -1426,392 +1429,142 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="11.5" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12.6719" style="1" customWidth="1"/>
-    <col min="3" max="3" width="13.5" style="1" customWidth="1"/>
-    <col min="4" max="4" width="28.5" style="1" customWidth="1"/>
-    <col min="5" max="5" width="14.1719" style="1" customWidth="1"/>
-    <col min="6" max="11" width="8.85156" style="1" customWidth="1"/>
-    <col min="12" max="13" width="30" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.85156" style="1" customWidth="1"/>
+    <col min="1" max="1" width="15" style="1" customWidth="1"/>
+    <col min="2" max="2" width="26.6719" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.85156" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13.1719" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8.85156" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="8.85156" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="13.55" customHeight="1">
       <c r="A1" t="s" s="2">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="3">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s" s="3">
+      <c r="B1" t="s" s="2">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s" s="2">
         <v>2</v>
       </c>
-      <c r="D1" t="s" s="3">
+      <c r="D1" t="s" s="2">
         <v>3</v>
       </c>
-      <c r="E1" t="s" s="3">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s" s="3">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s" s="3">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s" s="3">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s" s="3">
-        <v>8</v>
-      </c>
-      <c r="J1" t="s" s="3">
-        <v>9</v>
-      </c>
-      <c r="K1" t="s" s="3">
-        <v>10</v>
-      </c>
-      <c r="L1" t="s" s="3">
-        <v>11</v>
-      </c>
-      <c r="M1" t="s" s="3">
-        <v>12</v>
-      </c>
+      <c r="E1" s="3"/>
     </row>
     <row r="2" ht="13.55" customHeight="1">
       <c r="A2" t="s" s="4">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="B2" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="C2" t="s" s="5">
-        <v>15</v>
-      </c>
-      <c r="D2" t="s" s="5">
-        <v>16</v>
-      </c>
-      <c r="E2" t="s" s="5">
-        <v>17</v>
-      </c>
-      <c r="F2" s="6">
-        <v>1</v>
-      </c>
-      <c r="G2" s="6">
-        <v>200</v>
-      </c>
-      <c r="H2" s="6">
-        <v>1</v>
-      </c>
-      <c r="I2" s="6">
-        <v>2</v>
-      </c>
-      <c r="J2" s="6">
-        <v>1</v>
-      </c>
-      <c r="K2" s="6">
-        <v>10</v>
-      </c>
-      <c r="L2" t="s" s="4">
-        <v>18</v>
-      </c>
-      <c r="M2" t="s" s="4">
-        <v>19</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="C2" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s" s="4">
+        <v>7</v>
+      </c>
+      <c r="E2" s="3"/>
     </row>
     <row r="3" ht="13.55" customHeight="1">
       <c r="A3" t="s" s="4">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="C3" t="s" s="5">
-        <v>15</v>
-      </c>
-      <c r="D3" t="s" s="5">
-        <v>21</v>
-      </c>
-      <c r="E3" t="s" s="5">
-        <v>22</v>
-      </c>
-      <c r="F3" s="6">
-        <v>1</v>
-      </c>
-      <c r="G3" s="6">
-        <v>150</v>
-      </c>
-      <c r="H3" s="6">
-        <v>1</v>
-      </c>
-      <c r="I3" s="6">
-        <v>3</v>
-      </c>
-      <c r="J3" s="6">
-        <v>1</v>
-      </c>
-      <c r="K3" s="6">
-        <v>15</v>
-      </c>
-      <c r="L3" s="7"/>
-      <c r="M3" t="s" s="4">
-        <v>19</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="C3" t="s" s="4">
+        <v>10</v>
+      </c>
+      <c r="D3" t="s" s="4">
+        <v>11</v>
+      </c>
+      <c r="E3" s="3"/>
     </row>
     <row r="4" ht="13.55" customHeight="1">
       <c r="A4" t="s" s="4">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s" s="4">
-        <v>24</v>
-      </c>
-      <c r="C4" t="s" s="5">
-        <v>25</v>
-      </c>
-      <c r="D4" t="s" s="5">
-        <v>26</v>
-      </c>
-      <c r="E4" t="s" s="5">
-        <v>27</v>
-      </c>
-      <c r="F4" s="6">
-        <v>1</v>
-      </c>
-      <c r="G4" s="6">
-        <v>300</v>
-      </c>
-      <c r="H4" s="6">
-        <v>1</v>
-      </c>
-      <c r="I4" s="6">
-        <v>4</v>
-      </c>
-      <c r="J4" s="6">
-        <v>1</v>
-      </c>
-      <c r="K4" s="6">
-        <v>20</v>
-      </c>
-      <c r="L4" t="s" s="4">
-        <v>28</v>
-      </c>
-      <c r="M4" t="s" s="4">
-        <v>29</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="C4" t="s" s="4">
+        <v>6</v>
+      </c>
+      <c r="D4" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="E4" s="3"/>
     </row>
     <row r="5" ht="13.55" customHeight="1">
       <c r="A5" t="s" s="4">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s" s="4">
-        <v>31</v>
-      </c>
-      <c r="C5" t="s" s="5">
-        <v>32</v>
-      </c>
-      <c r="D5" t="s" s="5">
-        <v>33</v>
-      </c>
-      <c r="E5" t="s" s="5">
-        <v>17</v>
-      </c>
-      <c r="F5" s="6">
-        <v>1</v>
-      </c>
-      <c r="G5" s="6">
-        <v>20</v>
-      </c>
-      <c r="H5" s="6">
-        <v>1</v>
-      </c>
-      <c r="I5" s="6">
-        <v>5</v>
-      </c>
-      <c r="J5" s="6">
-        <v>1</v>
-      </c>
-      <c r="K5" s="6">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s" s="4">
         <v>10</v>
       </c>
-      <c r="L5" s="7"/>
-      <c r="M5" t="s" s="4">
-        <v>29</v>
-      </c>
+      <c r="D5" t="s" s="4">
+        <v>7</v>
+      </c>
+      <c r="E5" s="3"/>
     </row>
     <row r="6" ht="13.55" customHeight="1">
       <c r="A6" t="s" s="4">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s" s="4">
-        <v>35</v>
-      </c>
-      <c r="C6" t="s" s="5">
-        <v>36</v>
-      </c>
-      <c r="D6" t="s" s="5">
-        <v>37</v>
-      </c>
-      <c r="E6" t="s" s="5">
-        <v>17</v>
-      </c>
-      <c r="F6" s="6">
-        <v>1</v>
-      </c>
-      <c r="G6" s="6">
+        <v>18</v>
+      </c>
+      <c r="C6" t="s" s="4">
         <v>10</v>
       </c>
-      <c r="H6" s="6">
-        <v>1</v>
-      </c>
-      <c r="I6" s="6">
-        <v>10</v>
-      </c>
-      <c r="J6" s="6">
-        <v>1</v>
-      </c>
-      <c r="K6" s="6">
-        <v>10</v>
-      </c>
-      <c r="L6" s="7"/>
-      <c r="M6" t="s" s="4">
-        <v>29</v>
-      </c>
+      <c r="D6" t="s" s="4">
+        <v>7</v>
+      </c>
+      <c r="E6" s="3"/>
     </row>
     <row r="7" ht="13.55" customHeight="1">
       <c r="A7" t="s" s="4">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s" s="4">
-        <v>35</v>
-      </c>
-      <c r="C7" t="s" s="5">
-        <v>36</v>
-      </c>
-      <c r="D7" t="s" s="5">
-        <v>39</v>
-      </c>
-      <c r="E7" t="s" s="5">
-        <v>27</v>
-      </c>
-      <c r="F7" s="6">
-        <v>1</v>
-      </c>
-      <c r="G7" s="6">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s" s="4">
         <v>10</v>
       </c>
-      <c r="H7" s="6">
-        <v>1</v>
-      </c>
-      <c r="I7" s="6">
-        <v>10</v>
-      </c>
-      <c r="J7" s="6">
-        <v>1</v>
-      </c>
-      <c r="K7" s="6">
-        <v>10</v>
-      </c>
-      <c r="L7" s="7"/>
-      <c r="M7" t="s" s="4">
-        <v>19</v>
-      </c>
+      <c r="D7" t="s" s="4">
+        <v>7</v>
+      </c>
+      <c r="E7" s="3"/>
     </row>
     <row r="8" ht="13.55" customHeight="1">
-      <c r="A8" t="s" s="4">
-        <v>40</v>
-      </c>
-      <c r="B8" t="s" s="4">
-        <v>24</v>
-      </c>
-      <c r="C8" t="s" s="5">
-        <v>25</v>
-      </c>
-      <c r="D8" t="s" s="5">
-        <v>41</v>
-      </c>
-      <c r="E8" t="s" s="5">
-        <v>17</v>
-      </c>
-      <c r="F8" s="6">
-        <v>1</v>
-      </c>
-      <c r="G8" s="6">
-        <v>25</v>
-      </c>
-      <c r="H8" s="6">
-        <v>1</v>
-      </c>
-      <c r="I8" s="6">
-        <v>10</v>
-      </c>
-      <c r="J8" s="6">
-        <v>1</v>
-      </c>
-      <c r="K8" s="6">
-        <v>15</v>
-      </c>
-      <c r="L8" s="7"/>
-      <c r="M8" t="s" s="4">
-        <v>29</v>
-      </c>
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
     </row>
     <row r="9" ht="13.55" customHeight="1">
-      <c r="A9" t="s" s="4">
-        <v>42</v>
-      </c>
-      <c r="B9" t="s" s="4">
-        <v>43</v>
-      </c>
-      <c r="C9" t="s" s="4">
-        <v>44</v>
-      </c>
-      <c r="D9" t="s" s="4">
-        <v>45</v>
-      </c>
-      <c r="E9" t="s" s="4">
-        <v>22</v>
-      </c>
-      <c r="F9" s="8">
-        <v>1</v>
-      </c>
-      <c r="G9" s="8">
-        <v>15</v>
-      </c>
-      <c r="H9" s="8">
-        <v>1</v>
-      </c>
-      <c r="I9" s="8">
-        <v>10</v>
-      </c>
-      <c r="J9" s="8">
-        <v>1</v>
-      </c>
-      <c r="K9" s="8">
-        <v>20</v>
-      </c>
-      <c r="L9" t="s" s="4">
-        <v>28</v>
-      </c>
-      <c r="M9" t="s" s="4">
-        <v>19</v>
-      </c>
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
     </row>
     <row r="10" ht="13.55" customHeight="1">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
-      <c r="J10" s="7"/>
-      <c r="K10" s="7"/>
-      <c r="L10" s="7"/>
-      <c r="M10" s="7"/>
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1824,134 +1577,402 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="15" style="9" customWidth="1"/>
-    <col min="2" max="2" width="26.6719" style="9" customWidth="1"/>
-    <col min="3" max="3" width="8.85156" style="9" customWidth="1"/>
-    <col min="4" max="4" width="12.6719" style="9" customWidth="1"/>
-    <col min="5" max="5" width="8.85156" style="9" customWidth="1"/>
-    <col min="6" max="16384" width="8.85156" style="9" customWidth="1"/>
+    <col min="1" max="1" width="11.5" style="5" customWidth="1"/>
+    <col min="2" max="2" width="12.6719" style="5" customWidth="1"/>
+    <col min="3" max="3" width="13.5" style="5" customWidth="1"/>
+    <col min="4" max="4" width="28.5" style="5" customWidth="1"/>
+    <col min="5" max="5" width="14.1719" style="5" customWidth="1"/>
+    <col min="6" max="11" width="8.85156" style="5" customWidth="1"/>
+    <col min="12" max="13" width="30" style="5" customWidth="1"/>
+    <col min="14" max="16384" width="8.85156" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13.55" customHeight="1">
-      <c r="A1" t="s" s="10">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" t="s" s="6">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="10">
+      <c r="B1" t="s" s="7">
+        <v>21</v>
+      </c>
+      <c r="C1" t="s" s="7">
+        <v>22</v>
+      </c>
+      <c r="D1" t="s" s="7">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s" s="7">
+        <v>23</v>
+      </c>
+      <c r="F1" t="s" s="7">
+        <v>24</v>
+      </c>
+      <c r="G1" t="s" s="7">
+        <v>25</v>
+      </c>
+      <c r="H1" t="s" s="7">
+        <v>26</v>
+      </c>
+      <c r="I1" t="s" s="7">
+        <v>27</v>
+      </c>
+      <c r="J1" t="s" s="7">
+        <v>28</v>
+      </c>
+      <c r="K1" t="s" s="7">
+        <v>29</v>
+      </c>
+      <c r="L1" t="s" s="7">
         <v>3</v>
       </c>
-      <c r="C1" t="s" s="10">
-        <v>12</v>
-      </c>
-      <c r="D1" t="s" s="10">
-        <v>11</v>
-      </c>
-      <c r="E1" s="7"/>
+      <c r="M1" t="s" s="7">
+        <v>2</v>
+      </c>
     </row>
     <row r="2" ht="13.55" customHeight="1">
       <c r="A2" t="s" s="4">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="B2" t="s" s="4">
-        <v>15</v>
-      </c>
-      <c r="C2" t="s" s="4">
-        <v>19</v>
-      </c>
-      <c r="D2" t="s" s="4">
-        <v>28</v>
-      </c>
-      <c r="E2" s="7"/>
+        <v>4</v>
+      </c>
+      <c r="C2" t="s" s="8">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s" s="8">
+        <v>31</v>
+      </c>
+      <c r="E2" t="s" s="8">
+        <v>32</v>
+      </c>
+      <c r="F2" s="9">
+        <v>1</v>
+      </c>
+      <c r="G2" s="9">
+        <v>200</v>
+      </c>
+      <c r="H2" s="9">
+        <v>1</v>
+      </c>
+      <c r="I2" s="9">
+        <v>2</v>
+      </c>
+      <c r="J2" s="9">
+        <v>1</v>
+      </c>
+      <c r="K2" s="9">
+        <v>10</v>
+      </c>
+      <c r="L2" t="s" s="4">
+        <v>11</v>
+      </c>
+      <c r="M2" t="s" s="4">
+        <v>6</v>
+      </c>
     </row>
     <row r="3" ht="13.55" customHeight="1">
       <c r="A3" t="s" s="4">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="B3" t="s" s="4">
-        <v>25</v>
-      </c>
-      <c r="C3" t="s" s="4">
-        <v>29</v>
-      </c>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
+        <v>4</v>
+      </c>
+      <c r="C3" t="s" s="8">
+        <v>5</v>
+      </c>
+      <c r="D3" t="s" s="8">
+        <v>34</v>
+      </c>
+      <c r="E3" t="s" s="8">
+        <v>35</v>
+      </c>
+      <c r="F3" s="9">
+        <v>1</v>
+      </c>
+      <c r="G3" s="9">
+        <v>150</v>
+      </c>
+      <c r="H3" s="9">
+        <v>1</v>
+      </c>
+      <c r="I3" s="9">
+        <v>3</v>
+      </c>
+      <c r="J3" s="9">
+        <v>1</v>
+      </c>
+      <c r="K3" s="9">
+        <v>15</v>
+      </c>
+      <c r="L3" t="s" s="4">
+        <v>14</v>
+      </c>
+      <c r="M3" t="s" s="4">
+        <v>6</v>
+      </c>
     </row>
     <row r="4" ht="13.55" customHeight="1">
       <c r="A4" t="s" s="4">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="B4" t="s" s="4">
-        <v>32</v>
-      </c>
-      <c r="C4" t="s" s="4">
-        <v>19</v>
-      </c>
-      <c r="D4" t="s" s="4">
-        <v>46</v>
-      </c>
-      <c r="E4" s="7"/>
+        <v>8</v>
+      </c>
+      <c r="C4" t="s" s="8">
+        <v>9</v>
+      </c>
+      <c r="D4" t="s" s="8">
+        <v>37</v>
+      </c>
+      <c r="E4" t="s" s="8">
+        <v>38</v>
+      </c>
+      <c r="F4" s="9">
+        <v>1</v>
+      </c>
+      <c r="G4" s="9">
+        <v>300</v>
+      </c>
+      <c r="H4" s="9">
+        <v>1</v>
+      </c>
+      <c r="I4" s="9">
+        <v>4</v>
+      </c>
+      <c r="J4" s="9">
+        <v>1</v>
+      </c>
+      <c r="K4" s="9">
+        <v>20</v>
+      </c>
+      <c r="L4" t="s" s="4">
+        <v>7</v>
+      </c>
+      <c r="M4" t="s" s="4">
+        <v>10</v>
+      </c>
     </row>
     <row r="5" ht="13.55" customHeight="1">
       <c r="A5" t="s" s="4">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B5" t="s" s="4">
-        <v>36</v>
-      </c>
-      <c r="C5" t="s" s="4">
-        <v>29</v>
-      </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
+        <v>12</v>
+      </c>
+      <c r="C5" t="s" s="8">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s" s="8">
+        <v>40</v>
+      </c>
+      <c r="E5" t="s" s="8">
+        <v>32</v>
+      </c>
+      <c r="F5" s="9">
+        <v>1</v>
+      </c>
+      <c r="G5" s="9">
+        <v>20</v>
+      </c>
+      <c r="H5" s="9">
+        <v>1</v>
+      </c>
+      <c r="I5" s="9">
+        <v>5</v>
+      </c>
+      <c r="J5" s="9">
+        <v>1</v>
+      </c>
+      <c r="K5" s="9">
+        <v>10</v>
+      </c>
+      <c r="L5" t="s" s="4">
+        <v>7</v>
+      </c>
+      <c r="M5" t="s" s="4">
+        <v>10</v>
+      </c>
     </row>
     <row r="6" ht="13.55" customHeight="1">
       <c r="A6" t="s" s="4">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="B6" t="s" s="4">
-        <v>48</v>
-      </c>
-      <c r="C6" t="s" s="4">
-        <v>29</v>
-      </c>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
+        <v>15</v>
+      </c>
+      <c r="C6" t="s" s="8">
+        <v>16</v>
+      </c>
+      <c r="D6" t="s" s="8">
+        <v>42</v>
+      </c>
+      <c r="E6" t="s" s="8">
+        <v>32</v>
+      </c>
+      <c r="F6" s="9">
+        <v>1</v>
+      </c>
+      <c r="G6" s="9">
+        <v>10</v>
+      </c>
+      <c r="H6" s="9">
+        <v>1</v>
+      </c>
+      <c r="I6" s="9">
+        <v>10</v>
+      </c>
+      <c r="J6" s="9">
+        <v>1</v>
+      </c>
+      <c r="K6" s="9">
+        <v>10</v>
+      </c>
+      <c r="L6" t="s" s="4">
+        <v>7</v>
+      </c>
+      <c r="M6" t="s" s="4">
+        <v>10</v>
+      </c>
     </row>
     <row r="7" ht="13.55" customHeight="1">
       <c r="A7" t="s" s="4">
         <v>43</v>
       </c>
       <c r="B7" t="s" s="4">
+        <v>15</v>
+      </c>
+      <c r="C7" t="s" s="8">
+        <v>16</v>
+      </c>
+      <c r="D7" t="s" s="8">
+        <v>44</v>
+      </c>
+      <c r="E7" t="s" s="8">
+        <v>38</v>
+      </c>
+      <c r="F7" s="9">
+        <v>1</v>
+      </c>
+      <c r="G7" s="9">
+        <v>10</v>
+      </c>
+      <c r="H7" s="9">
+        <v>1</v>
+      </c>
+      <c r="I7" s="9">
+        <v>10</v>
+      </c>
+      <c r="J7" s="9">
+        <v>1</v>
+      </c>
+      <c r="K7" s="9">
+        <v>10</v>
+      </c>
+      <c r="L7" t="s" s="4">
+        <v>7</v>
+      </c>
+      <c r="M7" t="s" s="4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" ht="13.55" customHeight="1">
+      <c r="A8" t="s" s="4">
+        <v>45</v>
+      </c>
+      <c r="B8" t="s" s="4">
+        <v>8</v>
+      </c>
+      <c r="C8" t="s" s="8">
+        <v>9</v>
+      </c>
+      <c r="D8" t="s" s="8">
+        <v>46</v>
+      </c>
+      <c r="E8" t="s" s="8">
+        <v>32</v>
+      </c>
+      <c r="F8" s="9">
+        <v>1</v>
+      </c>
+      <c r="G8" s="9">
+        <v>25</v>
+      </c>
+      <c r="H8" s="9">
+        <v>1</v>
+      </c>
+      <c r="I8" s="9">
+        <v>10</v>
+      </c>
+      <c r="J8" s="9">
+        <v>1</v>
+      </c>
+      <c r="K8" s="9">
+        <v>15</v>
+      </c>
+      <c r="L8" t="s" s="4">
+        <v>7</v>
+      </c>
+      <c r="M8" t="s" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" ht="13.55" customHeight="1">
+      <c r="A9" t="s" s="4">
+        <v>47</v>
+      </c>
+      <c r="B9" t="s" s="4">
+        <v>19</v>
+      </c>
+      <c r="C9" t="s" s="4">
+        <v>48</v>
+      </c>
+      <c r="D9" t="s" s="4">
         <v>49</v>
       </c>
-      <c r="C7" t="s" s="4">
-        <v>29</v>
-      </c>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-    </row>
-    <row r="8" ht="13.55" customHeight="1">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-    </row>
-    <row r="9" ht="13.55" customHeight="1">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
+      <c r="E9" t="s" s="4">
+        <v>35</v>
+      </c>
+      <c r="F9" s="10">
+        <v>1</v>
+      </c>
+      <c r="G9" s="10">
+        <v>15</v>
+      </c>
+      <c r="H9" s="10">
+        <v>1</v>
+      </c>
+      <c r="I9" s="10">
+        <v>10</v>
+      </c>
+      <c r="J9" s="10">
+        <v>1</v>
+      </c>
+      <c r="K9" s="10">
+        <v>20</v>
+      </c>
+      <c r="L9" t="s" s="4">
+        <v>7</v>
+      </c>
+      <c r="M9" t="s" s="4">
+        <v>6</v>
+      </c>
     </row>
     <row r="10" ht="13.55" customHeight="1">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+      <c r="M10" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1964,7 +1985,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="15.5" style="11" customWidth="1"/>
@@ -1979,8 +2000,8 @@
     <col min="10" max="11" width="11.5" style="11" customWidth="1"/>
     <col min="12" max="12" width="15.5" style="11" customWidth="1"/>
     <col min="13" max="13" width="13.1719" style="11" customWidth="1"/>
-    <col min="14" max="15" width="24.8516" style="11" customWidth="1"/>
-    <col min="16" max="16384" width="8.85156" style="11" customWidth="1"/>
+    <col min="14" max="16" width="24.8516" style="11" customWidth="1"/>
+    <col min="17" max="16384" width="8.85156" style="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="13.55" customHeight="1">
@@ -1988,13 +2009,13 @@
         <v>0</v>
       </c>
       <c r="B1" t="s" s="4">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="C1" t="s" s="4">
         <v>50</v>
       </c>
       <c r="D1" t="s" s="12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E1" t="s" s="4">
         <v>51</v>
@@ -2027,7 +2048,10 @@
         <v>60</v>
       </c>
       <c r="O1" t="s" s="4">
-        <v>12</v>
+        <v>2</v>
+      </c>
+      <c r="P1" t="s" s="13">
+        <v>3</v>
       </c>
     </row>
     <row r="2" ht="90" customHeight="1">
@@ -2035,15 +2059,15 @@
         <v>61</v>
       </c>
       <c r="B2" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="C2" s="8">
+        <v>4</v>
+      </c>
+      <c r="C2" s="10">
         <v>2</v>
       </c>
       <c r="D2" t="s" s="12">
         <v>62</v>
       </c>
-      <c r="E2" s="8">
+      <c r="E2" s="10">
         <v>1</v>
       </c>
       <c r="F2" t="s" s="4">
@@ -2064,17 +2088,20 @@
       <c r="K2" t="s" s="4">
         <v>67</v>
       </c>
-      <c r="L2" t="b" s="8">
-        <v>1</v>
-      </c>
-      <c r="M2" t="b" s="8">
-        <v>1</v>
-      </c>
-      <c r="N2" t="b" s="8">
+      <c r="L2" t="b" s="10">
+        <v>1</v>
+      </c>
+      <c r="M2" t="b" s="10">
+        <v>1</v>
+      </c>
+      <c r="N2" t="b" s="10">
         <v>1</v>
       </c>
       <c r="O2" t="s" s="4">
-        <v>29</v>
+        <v>10</v>
+      </c>
+      <c r="P2" t="s" s="4">
+        <v>7</v>
       </c>
     </row>
     <row r="3" ht="105" customHeight="1">
@@ -2082,15 +2109,15 @@
         <v>68</v>
       </c>
       <c r="B3" t="s" s="4">
-        <v>14</v>
-      </c>
-      <c r="C3" s="8">
+        <v>4</v>
+      </c>
+      <c r="C3" s="10">
         <v>3</v>
       </c>
       <c r="D3" t="s" s="12">
         <v>69</v>
       </c>
-      <c r="E3" s="8">
+      <c r="E3" s="10">
         <v>2</v>
       </c>
       <c r="F3" t="s" s="4">
@@ -2111,17 +2138,20 @@
       <c r="K3" t="s" s="4">
         <v>67</v>
       </c>
-      <c r="L3" t="b" s="8">
-        <v>1</v>
-      </c>
-      <c r="M3" t="b" s="8">
+      <c r="L3" t="b" s="10">
+        <v>1</v>
+      </c>
+      <c r="M3" t="b" s="10">
         <v>0</v>
       </c>
-      <c r="N3" t="b" s="8">
+      <c r="N3" t="b" s="10">
         <v>1</v>
       </c>
       <c r="O3" t="s" s="4">
-        <v>19</v>
+        <v>6</v>
+      </c>
+      <c r="P3" t="s" s="4">
+        <v>7</v>
       </c>
     </row>
     <row r="4" ht="60" customHeight="1">
@@ -2129,15 +2159,15 @@
         <v>71</v>
       </c>
       <c r="B4" t="s" s="4">
-        <v>24</v>
-      </c>
-      <c r="C4" s="8">
+        <v>8</v>
+      </c>
+      <c r="C4" s="10">
         <v>4</v>
       </c>
       <c r="D4" t="s" s="12">
         <v>72</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="10">
         <v>3</v>
       </c>
       <c r="F4" t="s" s="4">
@@ -2158,17 +2188,20 @@
       <c r="K4" t="s" s="4">
         <v>67</v>
       </c>
-      <c r="L4" t="b" s="8">
+      <c r="L4" t="b" s="10">
         <v>0</v>
       </c>
-      <c r="M4" t="b" s="8">
-        <v>1</v>
-      </c>
-      <c r="N4" t="b" s="8">
+      <c r="M4" t="b" s="10">
+        <v>1</v>
+      </c>
+      <c r="N4" t="b" s="10">
         <v>0</v>
       </c>
       <c r="O4" t="s" s="4">
-        <v>19</v>
+        <v>6</v>
+      </c>
+      <c r="P4" t="s" s="4">
+        <v>7</v>
       </c>
     </row>
     <row r="5" ht="60" customHeight="1">
@@ -2176,15 +2209,15 @@
         <v>75</v>
       </c>
       <c r="B5" t="s" s="4">
-        <v>24</v>
-      </c>
-      <c r="C5" s="8">
+        <v>8</v>
+      </c>
+      <c r="C5" s="10">
         <v>5</v>
       </c>
       <c r="D5" t="s" s="12">
         <v>76</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="10">
         <v>4</v>
       </c>
       <c r="F5" t="s" s="4">
@@ -2205,17 +2238,20 @@
       <c r="K5" t="s" s="4">
         <v>67</v>
       </c>
-      <c r="L5" t="b" s="8">
-        <v>1</v>
-      </c>
-      <c r="M5" t="b" s="8">
-        <v>1</v>
-      </c>
-      <c r="N5" t="b" s="8">
+      <c r="L5" t="b" s="10">
+        <v>1</v>
+      </c>
+      <c r="M5" t="b" s="10">
+        <v>1</v>
+      </c>
+      <c r="N5" t="b" s="10">
         <v>1</v>
       </c>
       <c r="O5" t="s" s="4">
-        <v>29</v>
+        <v>10</v>
+      </c>
+      <c r="P5" t="s" s="4">
+        <v>7</v>
       </c>
     </row>
     <row r="6" ht="105" customHeight="1">
@@ -2223,18 +2259,18 @@
         <v>77</v>
       </c>
       <c r="B6" t="s" s="4">
-        <v>24</v>
-      </c>
-      <c r="C6" s="8">
+        <v>8</v>
+      </c>
+      <c r="C6" s="10">
         <v>5</v>
       </c>
       <c r="D6" t="s" s="12">
         <v>78</v>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="10">
         <v>5</v>
       </c>
-      <c r="F6" s="7"/>
+      <c r="F6" s="3"/>
       <c r="G6" t="s" s="4">
         <v>64</v>
       </c>
@@ -2250,17 +2286,20 @@
       <c r="K6" t="s" s="4">
         <v>67</v>
       </c>
-      <c r="L6" t="b" s="8">
-        <v>1</v>
-      </c>
-      <c r="M6" t="b" s="8">
-        <v>1</v>
-      </c>
-      <c r="N6" t="b" s="8">
+      <c r="L6" t="b" s="10">
+        <v>1</v>
+      </c>
+      <c r="M6" t="b" s="10">
+        <v>1</v>
+      </c>
+      <c r="N6" t="b" s="10">
         <v>1</v>
       </c>
       <c r="O6" t="s" s="4">
-        <v>29</v>
+        <v>10</v>
+      </c>
+      <c r="P6" t="s" s="4">
+        <v>7</v>
       </c>
     </row>
     <row r="7" ht="105" customHeight="1">
@@ -2268,22 +2307,22 @@
         <v>79</v>
       </c>
       <c r="B7" t="s" s="4">
-        <v>24</v>
-      </c>
-      <c r="C7" s="8">
+        <v>8</v>
+      </c>
+      <c r="C7" s="10">
         <v>5</v>
       </c>
       <c r="D7" t="s" s="12">
         <v>80</v>
       </c>
-      <c r="E7" s="8">
+      <c r="E7" s="10">
         <v>6</v>
       </c>
       <c r="F7" t="s" s="4">
         <v>63</v>
       </c>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
       <c r="I7" t="s" s="12">
         <v>70</v>
       </c>
@@ -2293,69 +2332,75 @@
       <c r="K7" t="s" s="4">
         <v>67</v>
       </c>
-      <c r="L7" t="b" s="8">
-        <v>1</v>
-      </c>
-      <c r="M7" t="b" s="8">
-        <v>1</v>
-      </c>
-      <c r="N7" t="b" s="8">
+      <c r="L7" t="b" s="10">
+        <v>1</v>
+      </c>
+      <c r="M7" t="b" s="10">
+        <v>1</v>
+      </c>
+      <c r="N7" t="b" s="10">
         <v>1</v>
       </c>
       <c r="O7" t="s" s="4">
-        <v>29</v>
+        <v>10</v>
+      </c>
+      <c r="P7" t="s" s="4">
+        <v>7</v>
       </c>
     </row>
     <row r="8" ht="13.55" customHeight="1">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
-      <c r="J8" s="7"/>
-      <c r="K8" s="7"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="7"/>
-      <c r="N8" s="7"/>
-      <c r="O8" s="7"/>
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="14"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3"/>
     </row>
     <row r="9" ht="13.55" customHeight="1">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
-      <c r="J9" s="7"/>
-      <c r="K9" s="7"/>
-      <c r="L9" s="7"/>
-      <c r="M9" s="7"/>
-      <c r="N9" s="7"/>
-      <c r="O9" s="7"/>
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="3"/>
+      <c r="O9" s="3"/>
+      <c r="P9" s="3"/>
     </row>
     <row r="10" ht="13.55" customHeight="1">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
-      <c r="J10" s="7"/>
-      <c r="K10" s="7"/>
-      <c r="L10" s="7"/>
-      <c r="M10" s="7"/>
-      <c r="N10" s="7"/>
-      <c r="O10" s="7"/>
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="3"/>
+      <c r="O10" s="3"/>
+      <c r="P10" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
rollback seed from changes column of SeedVersion Table
</commit_message>
<xml_diff>
--- a/src/seed/seed-data/excel/data-seed.xlsx
+++ b/src/seed/seed-data/excel/data-seed.xlsx
@@ -75,7 +75,7 @@
     <t>ind_uid_6</t>
   </si>
   <si>
-    <t>Footwear</t>
+    <t>Footwear Technology</t>
   </si>
   <si>
     <t>industryId</t>
@@ -141,13 +141,13 @@
     <t>temp_uid_5</t>
   </si>
   <si>
-    <t>Fusing machine</t>
+    <t>Fusing machine Template</t>
   </si>
   <si>
     <t>temp_uid_6</t>
   </si>
   <si>
-    <t>Knitting machine</t>
+    <t>Knitting machine Template</t>
   </si>
   <si>
     <t>temp_uid_7</t>
@@ -1429,7 +1429,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="15" style="1" customWidth="1"/>
@@ -1559,13 +1559,6 @@
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" ht="13.55" customHeight="1">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>
@@ -1577,7 +1570,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="11.5" style="5" customWidth="1"/>
@@ -1874,7 +1867,7 @@
         <v>7</v>
       </c>
       <c r="M7" t="s" s="4">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" ht="13.55" customHeight="1">
@@ -1958,21 +1951,6 @@
       <c r="M9" t="s" s="4">
         <v>6</v>
       </c>
-    </row>
-    <row r="10" ht="13.55" customHeight="1">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>